<commit_message>
Actualizacion automatica 2026-09-15 17:38 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -6770,7 +6770,7 @@
         <v>46195.50768850694</v>
       </c>
       <c r="D86" s="5">
-        <v>46272.13737606481</v>
+        <v>46280.1264971412</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>272</v>
@@ -6814,8 +6814,8 @@
       <c r="R86" s="5">
         <v>46279</v>
       </c>
-      <c r="S86" s="12" t="s">
-        <v>74</v>
+      <c r="S86" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T86" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-16 17:36 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -7450,7 +7450,7 @@
         <v>46196.76839824074</v>
       </c>
       <c r="D98" s="5">
-        <v>46228.10704425926</v>
+        <v>46281.12945644676</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>291</v>
@@ -7494,8 +7494,8 @@
       <c r="R98" s="5">
         <v>46288</v>
       </c>
-      <c r="S98" s="11" t="s">
-        <v>107</v>
+      <c r="S98" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="T98" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-09-18 17:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001466 - ZITRON PERU PODEROSA.xlsx
+++ b/data/50001466 - ZITRON PERU PODEROSA.xlsx
@@ -7110,7 +7110,7 @@
         <v>46196.76755512731</v>
       </c>
       <c r="D92" s="5">
-        <v>46275.15928740741</v>
+        <v>46283.1630549074</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>281</v>
@@ -7154,8 +7154,8 @@
       <c r="R92" s="5">
         <v>46282</v>
       </c>
-      <c r="S92" s="12" t="s">
-        <v>74</v>
+      <c r="S92" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T92" s="6">
         <v>1</v>

</xml_diff>